<commit_message>
replace Molex 502774-0891 with GCT MEM2052-00-195-00-A
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Hardware_projects\MusselGapeTracker_hardware\KiCad_files\MusselGapeTracker_RevH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wmedu-my.sharepoint.com/personal/joslater_wm_edu/Documents/VIMS/aubrey_project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD93A51B-BD97-4CA2-B6E7-B1695BBF3334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{AB5E46A4-20F2-224B-A54B-BAAB896D7AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1DC8607-A9B0-004D-BB5D-A2F480AC0CD8}"/>
   <bookViews>
-    <workbookView xWindow="-34000" yWindow="830" windowWidth="23270" windowHeight="19070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MusselGapeTracker_RevH" sheetId="2" r:id="rId1"/>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="439">
   <si>
     <t>Part Description</t>
   </si>
@@ -456,9 +456,6 @@
     <t>(3 boards for this price)</t>
   </si>
   <si>
-    <t>(varies based on length needs)</t>
-  </si>
-  <si>
     <t>Subtotal</t>
   </si>
   <si>
@@ -963,15 +960,6 @@
     <t>CKN9104CT-ND</t>
   </si>
   <si>
-    <t>490-10728-1-ND</t>
-  </si>
-  <si>
-    <t>GRM188R61C106KAALD</t>
-  </si>
-  <si>
-    <t>Murata</t>
-  </si>
-  <si>
     <t>Capacitor, 0603 10µF X5R</t>
   </si>
   <si>
@@ -1326,21 +1314,9 @@
     <t>296-31822-1-ND</t>
   </si>
   <si>
-    <t>74HC4067PW,118</t>
-  </si>
-  <si>
-    <t>1727-2042-1-ND</t>
-  </si>
-  <si>
-    <t>74HC4067PW,118 multiplexer 16 channel (24-TSSOP 4.4x7.8mm, 0.65mm pitch)</t>
-  </si>
-  <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>*changed from prior revision</t>
-  </si>
-  <si>
     <t>ATMEGA328P-AURCT-ND</t>
   </si>
   <si>
@@ -1393,6 +1369,49 @@
   </si>
   <si>
     <t xml:space="preserve">O-ring 1/8 width dash number 206 - McMasterCarr pk 100 https://www.mcmaster.com/4061t228/ </t>
+  </si>
+  <si>
+    <t>CC0603KRX5R7BB106</t>
+  </si>
+  <si>
+    <t>311-3486-2-ND</t>
+  </si>
+  <si>
+    <t>FIND SUBSTITUTE</t>
+  </si>
+  <si>
+    <t>slater substitute</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">(varies based on length needs), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>FIND SUBSTITUTE</t>
+    </r>
+  </si>
+  <si>
+    <t>CD74HC4067PWR multiplexer 16 channel (24-TSSOP 4.4x7.8mm, 0.65mm pitch)</t>
+  </si>
+  <si>
+    <t>CD74HC4067PWR</t>
+  </si>
+  <si>
+    <t>296-CD74HC4067PWRCT-ND</t>
+  </si>
+  <si>
+    <t>FIND SUBSTITUTE, OR AVAILABLE AT https://www.lcsc.com/product-detail/C131334.html</t>
+  </si>
+  <si>
+    <t>USE ALT</t>
+  </si>
+  <si>
+    <t>NEED SUB IF USING DIFF HEADER</t>
   </si>
 </sst>
 </file>
@@ -1404,7 +1423,7 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1476,6 +1495,18 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1554,7 +1585,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1631,10 +1662,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2000,25 +2037,28 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M74"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M84"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="52.36328125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="23.81640625" customWidth="1"/>
-    <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.1796875" style="7" customWidth="1"/>
-    <col min="6" max="6" width="19.453125" customWidth="1"/>
-    <col min="7" max="7" width="10.453125" style="6" customWidth="1"/>
-    <col min="8" max="8" width="12.36328125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="52.33203125" style="4" customWidth="1"/>
+    <col min="2" max="2" width="23.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.1640625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="19.5" customWidth="1"/>
+    <col min="7" max="7" width="10.5" style="6" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="23.5" customWidth="1"/>
+    <col min="10" max="10" width="18.33203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" s="15" customFormat="1" x14ac:dyDescent="0.35">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" s="15" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
@@ -2044,22 +2084,22 @@
         <v>12</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="J2" s="15" t="s">
+        <v>344</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>345</v>
+      </c>
+      <c r="L2" s="15" t="s">
         <v>348</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="M2" s="15" t="s">
         <v>349</v>
       </c>
-      <c r="L2" s="15" t="s">
-        <v>352</v>
-      </c>
-      <c r="M2" s="15" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -2079,14 +2119,14 @@
         <v>11</v>
       </c>
       <c r="G3" s="5">
-        <v>0.46</v>
+        <v>0.38</v>
       </c>
       <c r="H3" s="6">
         <f>G3*E3</f>
-        <v>0.92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>13</v>
       </c>
@@ -2106,16 +2146,16 @@
         <v>17</v>
       </c>
       <c r="G4" s="6">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="H4" s="6">
         <f>G4*E4</f>
-        <v>2.4000000000000004</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -2124,50 +2164,53 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E5" s="7">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G5" s="6">
-        <v>0.17</v>
+        <v>0.73</v>
       </c>
       <c r="H5" s="6">
         <f>G5*E5</f>
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>295</v>
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="43" t="s">
+        <v>291</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>428</v>
       </c>
       <c r="E6" s="7">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>292</v>
+        <v>429</v>
       </c>
       <c r="G6" s="6">
-        <v>0.39</v>
+        <v>0.65</v>
       </c>
       <c r="H6" s="6">
         <f>G6*E6</f>
-        <v>0.39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.65</v>
+      </c>
+      <c r="I6" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -2194,7 +2237,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>115</v>
       </c>
@@ -2221,7 +2264,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>23</v>
       </c>
@@ -2248,7 +2291,7 @@
         <v>2.7</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>27</v>
       </c>
@@ -2275,7 +2318,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>26</v>
       </c>
@@ -2302,7 +2345,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
@@ -2322,14 +2365,14 @@
         <v>36</v>
       </c>
       <c r="G12" s="6">
-        <v>0.31</v>
+        <v>0.13</v>
       </c>
       <c r="H12" s="6">
         <f t="shared" si="0"/>
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -2349,53 +2392,53 @@
         <v>39</v>
       </c>
       <c r="G13" s="6">
-        <v>0.28999999999999998</v>
+        <v>0.12</v>
       </c>
       <c r="H13" s="6">
         <f t="shared" si="0"/>
-        <v>0.28999999999999998</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="D14" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="E14" s="7">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="G14" s="6">
-        <v>0.5</v>
+        <v>0.62</v>
       </c>
       <c r="H14" s="6">
         <f t="shared" si="0"/>
-        <v>0.5</v>
+        <v>0.62</v>
       </c>
       <c r="J14" t="s">
+        <v>346</v>
+      </c>
+      <c r="K14" t="s">
+        <v>347</v>
+      </c>
+      <c r="L14" t="s">
+        <v>351</v>
+      </c>
+      <c r="M14" t="s">
         <v>350</v>
       </c>
-      <c r="K14" t="s">
-        <v>351</v>
-      </c>
-      <c r="L14" t="s">
-        <v>355</v>
-      </c>
-      <c r="M14" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>41</v>
       </c>
@@ -2415,16 +2458,16 @@
         <v>45</v>
       </c>
       <c r="G15" s="6">
-        <v>0.82</v>
+        <v>0.59</v>
       </c>
       <c r="H15" s="6">
         <f t="shared" si="0"/>
-        <v>2.46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B16" t="s">
         <v>46</v>
@@ -2433,53 +2476,53 @@
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E16" s="7">
         <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="G16" s="6">
-        <v>2</v>
+        <v>1.22</v>
       </c>
       <c r="H16" s="6">
         <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+        <v>19.52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="E17" s="7">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>362</v>
+        <v>358</v>
       </c>
       <c r="G17" s="6">
-        <v>9.7100000000000009</v>
+        <v>12.46</v>
       </c>
       <c r="H17" s="6">
         <f t="shared" si="0"/>
-        <v>9.7100000000000009</v>
+        <v>12.46</v>
       </c>
       <c r="J17" t="s">
-        <v>422</v>
+        <v>414</v>
       </c>
       <c r="K17" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>49</v>
       </c>
@@ -2499,14 +2542,14 @@
         <v>52</v>
       </c>
       <c r="G18" s="6">
-        <v>0.57999999999999996</v>
+        <v>0.4</v>
       </c>
       <c r="H18" s="6">
         <f t="shared" si="0"/>
-        <v>0.57999999999999996</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>53</v>
       </c>
@@ -2514,23 +2557,23 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E19" s="7">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="G19" s="6">
-        <v>1</v>
+        <v>1.03</v>
       </c>
       <c r="H19" s="6">
         <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1.03</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>63</v>
       </c>
@@ -2556,8 +2599,11 @@
         <f t="shared" si="0"/>
         <v>3.84</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I20" s="39" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>66</v>
       </c>
@@ -2580,8 +2626,11 @@
         <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="I21" s="39" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>67</v>
       </c>
@@ -2598,20 +2647,21 @@
         <v>69</v>
       </c>
       <c r="G22" s="6">
-        <v>0.1</v>
+        <v>4.0899999999999999E-2</v>
       </c>
       <c r="H22" s="6">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
+        <v>4.09</v>
+      </c>
+      <c r="I22" s="39"/>
       <c r="J22" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="K22" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>59</v>
       </c>
@@ -2631,14 +2681,14 @@
         <v>62</v>
       </c>
       <c r="G23" s="6">
-        <v>0.6</v>
+        <v>0.37</v>
       </c>
       <c r="H23" s="6">
         <f t="shared" si="0"/>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>80</v>
       </c>
@@ -2655,14 +2705,14 @@
         <v>82</v>
       </c>
       <c r="G24" s="6">
-        <v>0.74</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="H24" s="6">
         <f t="shared" si="0"/>
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>83</v>
       </c>
@@ -2682,14 +2732,14 @@
         <v>87</v>
       </c>
       <c r="G25" s="6">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="H25" s="6">
         <f t="shared" si="0"/>
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>88</v>
       </c>
@@ -2709,16 +2759,16 @@
         <v>90</v>
       </c>
       <c r="G26" s="6">
-        <v>1.38</v>
+        <v>1.8</v>
       </c>
       <c r="H26" s="6">
         <f t="shared" si="0"/>
-        <v>1.38</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="B27" t="s">
         <v>92</v>
@@ -2736,20 +2786,20 @@
         <v>91</v>
       </c>
       <c r="G27" s="6">
-        <v>0.38</v>
+        <v>0.51</v>
       </c>
       <c r="H27" s="6">
         <f t="shared" si="0"/>
-        <v>0.38</v>
+        <v>0.51</v>
       </c>
       <c r="J27" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>95</v>
       </c>
@@ -2775,14 +2825,17 @@
         <f t="shared" si="0"/>
         <v>0.38</v>
       </c>
+      <c r="I28" s="40" t="s">
+        <v>437</v>
+      </c>
       <c r="J28" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="K28" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>101</v>
       </c>
@@ -2799,17 +2852,17 @@
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="G29" s="6">
-        <v>0.54</v>
+        <v>0.72</v>
       </c>
       <c r="H29" s="6">
         <f t="shared" si="0"/>
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>106</v>
       </c>
@@ -2835,35 +2888,38 @@
         <f t="shared" si="0"/>
         <v>3.64</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>415</v>
-      </c>
-      <c r="C31" s="37" t="s">
-        <v>97</v>
-      </c>
-      <c r="D31" s="37" t="s">
-        <v>413</v>
-      </c>
-      <c r="E31" s="38">
-        <v>1</v>
-      </c>
-      <c r="F31" s="37" t="s">
-        <v>414</v>
+      <c r="I30" s="39" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="37" t="s">
+        <v>433</v>
+      </c>
+      <c r="C31" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D31" s="41" t="s">
+        <v>434</v>
+      </c>
+      <c r="E31" s="42">
+        <v>1</v>
+      </c>
+      <c r="F31" s="41" t="s">
+        <v>435</v>
       </c>
       <c r="G31" s="6">
-        <v>1.19</v>
+        <v>1.25</v>
       </c>
       <c r="H31" s="6">
         <f t="shared" si="0"/>
-        <v>1.19</v>
-      </c>
-      <c r="I31" s="37" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1.25</v>
+      </c>
+      <c r="I31" s="41" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>108</v>
       </c>
@@ -2874,34 +2930,34 @@
         <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>419</v>
+        <v>411</v>
       </c>
       <c r="E32" s="7">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="G32" s="6">
-        <v>2.0699999999999998</v>
+        <v>2.74</v>
       </c>
       <c r="H32" s="6">
         <f t="shared" si="0"/>
-        <v>2.0699999999999998</v>
+        <v>2.74</v>
       </c>
       <c r="J32" t="s">
-        <v>421</v>
+        <v>413</v>
       </c>
       <c r="K32" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C33" t="s">
         <v>126</v>
-      </c>
-      <c r="C33" t="s">
-        <v>127</v>
       </c>
       <c r="D33">
         <v>8195</v>
@@ -2910,119 +2966,119 @@
         <v>16</v>
       </c>
       <c r="F33" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G33" s="6">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="H33" s="6">
         <f t="shared" si="0"/>
-        <v>3.68</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
         <v>129</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>130</v>
       </c>
-      <c r="D34" t="s">
+      <c r="E34" s="7">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
         <v>131</v>
       </c>
-      <c r="E34" s="7">
-        <v>1</v>
-      </c>
-      <c r="F34" t="s">
-        <v>132</v>
-      </c>
       <c r="G34" s="6">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="H34" s="6">
         <f t="shared" si="0"/>
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C35" t="s">
+        <v>315</v>
+      </c>
+      <c r="D35" t="s">
         <v>319</v>
       </c>
-      <c r="D35" t="s">
-        <v>323</v>
-      </c>
       <c r="E35" s="7">
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="G35" s="6">
-        <v>1.45</v>
+        <v>1.71</v>
       </c>
       <c r="H35" s="6">
         <f t="shared" si="0"/>
-        <v>1.45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+        <v>1.71</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
         <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E36" s="7">
         <v>1</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G36" s="6">
-        <v>0.83</v>
+        <v>0.64</v>
       </c>
       <c r="H36" s="6">
         <f t="shared" si="0"/>
-        <v>0.83</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B37" t="s">
         <v>288</v>
       </c>
-      <c r="B37" t="s">
+      <c r="D37" s="21" t="s">
         <v>289</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="E37" s="7">
+        <v>1</v>
+      </c>
+      <c r="F37" s="21" t="s">
         <v>290</v>
       </c>
-      <c r="E37" s="7">
-        <v>1</v>
-      </c>
-      <c r="F37" s="21" t="s">
-        <v>291</v>
-      </c>
       <c r="G37" s="6">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="H37" s="6">
         <f t="shared" si="0"/>
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>70</v>
       </c>
@@ -3049,10 +3105,10 @@
         <v>0.16</v>
       </c>
       <c r="I38" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>75</v>
       </c>
@@ -3069,17 +3125,17 @@
         <v>78</v>
       </c>
       <c r="G39" s="6">
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="H39" s="6">
         <f>G39*E39</f>
-        <v>0.17</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="I39" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>76</v>
       </c>
@@ -3096,255 +3152,75 @@
         <v>77</v>
       </c>
       <c r="G40" s="6">
-        <v>0.23</v>
+        <v>0.15</v>
       </c>
       <c r="H40" s="6">
         <f>G40*E40</f>
-        <v>2.3000000000000003</v>
+        <v>1.5</v>
       </c>
       <c r="I40" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="D41" s="21"/>
       <c r="F41" s="21"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G42" s="19" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H42" s="19">
         <f>SUM(H3:H37)</f>
-        <v>88.369999999999976</v>
+        <v>72.669999999999973</v>
       </c>
       <c r="I42" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>113</v>
       </c>
       <c r="C44" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D44" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="F44" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="H44" s="12">
         <v>4.62</v>
       </c>
       <c r="I44" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="H45" s="12"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A46" s="10" t="s">
-        <v>296</v>
-      </c>
-      <c r="H46" s="12"/>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A47" s="4" t="s">
-        <v>300</v>
-      </c>
-      <c r="C47" t="s">
-        <v>299</v>
-      </c>
-      <c r="D47" t="s">
-        <v>298</v>
-      </c>
-      <c r="E47" s="7">
-        <v>16</v>
-      </c>
-      <c r="F47" t="s">
-        <v>297</v>
-      </c>
-      <c r="G47" s="6">
-        <v>1.31</v>
-      </c>
-      <c r="H47" s="6">
-        <f t="shared" ref="H47:H52" si="1">G47*E47</f>
-        <v>20.96</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A48" s="4" t="s">
-        <v>306</v>
-      </c>
-      <c r="C48" t="s">
-        <v>305</v>
-      </c>
-      <c r="D48" t="s">
-        <v>307</v>
-      </c>
-      <c r="E48" s="7">
-        <v>1</v>
-      </c>
-      <c r="F48" t="s">
-        <v>308</v>
-      </c>
-      <c r="G48" s="6">
-        <v>18.28</v>
-      </c>
-      <c r="H48" s="6">
-        <f t="shared" si="1"/>
-        <v>18.28</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A49" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="C49" t="s">
-        <v>309</v>
-      </c>
-      <c r="D49" t="s">
-        <v>311</v>
-      </c>
-      <c r="E49" s="7">
-        <v>1</v>
-      </c>
-      <c r="F49" t="s">
-        <v>310</v>
-      </c>
-      <c r="G49" s="6">
-        <v>10.81</v>
-      </c>
-      <c r="H49" s="6">
-        <f t="shared" si="1"/>
-        <v>10.81</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A50" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="C50" t="s">
-        <v>309</v>
-      </c>
-      <c r="D50" t="s">
-        <v>313</v>
-      </c>
-      <c r="E50" s="7">
-        <v>1</v>
-      </c>
-      <c r="F50" t="s">
-        <v>314</v>
-      </c>
-      <c r="G50" s="6">
-        <v>7.8</v>
-      </c>
-      <c r="H50" s="6">
-        <f t="shared" si="1"/>
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="29" x14ac:dyDescent="0.35">
-      <c r="A51" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="C51" t="s">
-        <v>433</v>
-      </c>
-      <c r="D51" t="s">
-        <v>431</v>
-      </c>
-      <c r="E51">
-        <v>1</v>
-      </c>
-      <c r="F51" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A52" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="C52" t="s">
-        <v>327</v>
-      </c>
-      <c r="D52" t="s">
-        <v>328</v>
-      </c>
-      <c r="E52" s="7">
-        <v>1</v>
-      </c>
-      <c r="F52" t="s">
-        <v>329</v>
-      </c>
-      <c r="G52" s="6">
-        <v>2.19</v>
-      </c>
-      <c r="H52" s="6">
-        <f t="shared" si="1"/>
-        <v>2.19</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A53" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="C53" t="s">
-        <v>319</v>
-      </c>
-      <c r="D53" t="s">
-        <v>320</v>
-      </c>
-      <c r="E53" s="7">
-        <v>1</v>
-      </c>
-      <c r="F53" t="s">
-        <v>321</v>
-      </c>
-      <c r="G53" s="6">
-        <v>3.51</v>
-      </c>
-      <c r="H53" s="6">
-        <f>G53*E53</f>
-        <v>3.51</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="C54" t="s">
-        <v>434</v>
-      </c>
-      <c r="D54" t="s">
-        <v>434</v>
-      </c>
-      <c r="E54" s="7">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:11" ht="30.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="E57" s="7">
         <v>1</v>
@@ -3360,12 +3236,12 @@
         <v>122</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="E58" s="7">
         <v>16</v>
@@ -3377,25 +3253,25 @@
         <f>G58*E58</f>
         <v>8</v>
       </c>
-      <c r="K58" s="39"/>
-    </row>
-    <row r="59" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K58" s="38"/>
+    </row>
+    <row r="59" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C59" s="23"/>
       <c r="G59" s="11"/>
       <c r="H59" s="11"/>
     </row>
-    <row r="60" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
         <v>118</v>
       </c>
       <c r="G60" s="11"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="C61" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E61" s="7">
         <v>1</v>
@@ -3411,40 +3287,40 @@
         <v>121</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="C62" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="E62" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C63" s="23"/>
       <c r="G63" s="11"/>
       <c r="H63" s="11"/>
     </row>
-    <row r="64" spans="1:11" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
         <v>109</v>
       </c>
       <c r="E64"/>
       <c r="F64" s="9" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="E65" s="7">
         <v>1</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="G65" s="6">
         <v>9.99</v>
@@ -3454,7 +3330,7 @@
         <v>9.99</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>120</v>
       </c>
@@ -3468,32 +3344,32 @@
         <v>6.99</v>
       </c>
       <c r="H66" s="6">
-        <f t="shared" ref="H66" si="2">G66*E66</f>
+        <f t="shared" ref="H66" si="1">G66*E66</f>
         <v>6.99</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67"/>
       <c r="E67"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68"/>
       <c r="E68"/>
       <c r="G68" s="19" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>196.5866666666667</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+        <v>117.33666666666667</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="E69"/>
     </row>
-    <row r="70" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>110</v>
       </c>
@@ -3514,21 +3390,21 @@
         <v>121</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="C71" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="D71" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="E71" s="7">
         <v>1</v>
       </c>
       <c r="F71" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="G71" s="6">
         <v>64.5</v>
@@ -3537,48 +3413,229 @@
         <v>121</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="C72" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D72" t="s">
-        <v>346</v>
+        <v>342</v>
       </c>
       <c r="E72" s="7">
         <v>1</v>
       </c>
       <c r="F72" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="G72" s="6">
         <v>129.94999999999999</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C73" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="D73" t="s">
-        <v>347</v>
+        <v>343</v>
       </c>
       <c r="E73" s="7">
         <v>1</v>
       </c>
       <c r="F73" s="24" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="G73" s="6">
         <v>129</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G74" s="19"/>
+    </row>
+    <row r="76" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A76" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="H76" s="12"/>
+    </row>
+    <row r="77" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="C77" t="s">
+        <v>295</v>
+      </c>
+      <c r="D77" t="s">
+        <v>294</v>
+      </c>
+      <c r="E77" s="7">
+        <v>16</v>
+      </c>
+      <c r="F77" t="s">
+        <v>293</v>
+      </c>
+      <c r="G77" s="6">
+        <v>1.31</v>
+      </c>
+      <c r="H77" s="6">
+        <f t="shared" ref="H77:H82" si="2">G77*E77</f>
+        <v>20.96</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A78" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="C78" t="s">
+        <v>301</v>
+      </c>
+      <c r="D78" t="s">
+        <v>303</v>
+      </c>
+      <c r="E78" s="7">
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
+        <v>304</v>
+      </c>
+      <c r="G78" s="6">
+        <v>18.28</v>
+      </c>
+      <c r="H78" s="6">
+        <f t="shared" si="2"/>
+        <v>18.28</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A79" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="C79" t="s">
+        <v>305</v>
+      </c>
+      <c r="D79" t="s">
+        <v>307</v>
+      </c>
+      <c r="E79" s="7">
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
+        <v>306</v>
+      </c>
+      <c r="G79" s="6">
+        <v>10.81</v>
+      </c>
+      <c r="H79" s="6">
+        <f t="shared" si="2"/>
+        <v>10.81</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A80" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C80" t="s">
+        <v>305</v>
+      </c>
+      <c r="D80" t="s">
+        <v>309</v>
+      </c>
+      <c r="E80" s="7">
+        <v>1</v>
+      </c>
+      <c r="F80" t="s">
+        <v>310</v>
+      </c>
+      <c r="G80" s="6">
+        <v>7.8</v>
+      </c>
+      <c r="H80" s="6">
+        <f t="shared" si="2"/>
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A81" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="C81" t="s">
+        <v>425</v>
+      </c>
+      <c r="D81" t="s">
+        <v>423</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A82" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="C82" t="s">
+        <v>323</v>
+      </c>
+      <c r="D82" t="s">
+        <v>324</v>
+      </c>
+      <c r="E82" s="7">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
+        <v>325</v>
+      </c>
+      <c r="G82" s="6">
+        <v>2.19</v>
+      </c>
+      <c r="H82" s="6">
+        <f t="shared" si="2"/>
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A83" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="C83" t="s">
+        <v>315</v>
+      </c>
+      <c r="D83" t="s">
+        <v>316</v>
+      </c>
+      <c r="E83" s="7">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
+        <v>317</v>
+      </c>
+      <c r="G83" s="6">
+        <v>3.51</v>
+      </c>
+      <c r="H83" s="6">
+        <f>G83*E83</f>
+        <v>3.51</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="A84" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="C84" t="s">
+        <v>426</v>
+      </c>
+      <c r="D84" t="s">
+        <v>426</v>
+      </c>
+      <c r="E84" s="7">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B3">
@@ -3607,474 +3664,474 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.1796875" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1796875" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.1640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>197</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="C1" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C2" t="s">
         <v>200</v>
       </c>
-      <c r="D1" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="7">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="C2" t="s">
-        <v>201</v>
-      </c>
       <c r="D2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D3" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D4" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D5" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="7">
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D6" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="7">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D7" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="7">
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C8" t="s">
         <v>206</v>
       </c>
-      <c r="C8" t="s">
-        <v>207</v>
-      </c>
       <c r="D8" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="7">
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="C9" t="s">
         <v>208</v>
       </c>
-      <c r="C9" t="s">
-        <v>209</v>
-      </c>
       <c r="D9" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="7">
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="C10" t="s">
         <v>210</v>
       </c>
-      <c r="C10" t="s">
-        <v>211</v>
-      </c>
       <c r="D10" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="7">
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" t="s">
         <v>212</v>
       </c>
-      <c r="C11" t="s">
-        <v>213</v>
-      </c>
       <c r="D11" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="7">
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D12" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="7">
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C13" t="s">
         <v>216</v>
       </c>
-      <c r="C13" t="s">
-        <v>217</v>
-      </c>
       <c r="D13" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="7">
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" t="s">
         <v>218</v>
       </c>
-      <c r="C14" t="s">
-        <v>219</v>
-      </c>
       <c r="D14" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="7">
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="C15" t="s">
         <v>220</v>
       </c>
-      <c r="C15" t="s">
-        <v>221</v>
-      </c>
       <c r="D15" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="7">
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="C16" t="s">
         <v>222</v>
       </c>
-      <c r="C16" t="s">
-        <v>223</v>
-      </c>
       <c r="D16" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="7">
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C17" t="s">
         <v>224</v>
       </c>
-      <c r="C17" t="s">
-        <v>225</v>
-      </c>
       <c r="D17" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="7">
         <v>17</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C18" t="s">
         <v>226</v>
       </c>
-      <c r="C18" t="s">
-        <v>227</v>
-      </c>
       <c r="D18" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="7">
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D19" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="7">
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C20" t="s">
         <v>229</v>
       </c>
-      <c r="C20" t="s">
-        <v>230</v>
-      </c>
       <c r="D20" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="7">
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C21" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D21" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="7">
         <v>21</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C22" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D22" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="7">
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C23" t="s">
         <v>233</v>
       </c>
-      <c r="C23" t="s">
-        <v>234</v>
-      </c>
       <c r="D23" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="7">
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C24" t="s">
         <v>235</v>
       </c>
-      <c r="C24" t="s">
-        <v>236</v>
-      </c>
       <c r="D24" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="7">
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C25" t="s">
         <v>237</v>
       </c>
-      <c r="C25" t="s">
-        <v>238</v>
-      </c>
       <c r="D25" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="7">
         <v>25</v>
       </c>
       <c r="B26" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C26" t="s">
         <v>239</v>
       </c>
-      <c r="C26" t="s">
-        <v>240</v>
-      </c>
       <c r="D26" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="7">
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="C27" t="s">
         <v>241</v>
       </c>
-      <c r="C27" t="s">
-        <v>242</v>
-      </c>
       <c r="D27" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="7">
         <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="C28" t="s">
         <v>243</v>
       </c>
-      <c r="C28" t="s">
-        <v>244</v>
-      </c>
       <c r="D28" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="7">
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C29" t="s">
         <v>245</v>
       </c>
-      <c r="C29" t="s">
-        <v>246</v>
-      </c>
       <c r="D29" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="7">
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D30" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="7">
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>247</v>
+      </c>
+      <c r="C31" t="s">
         <v>248</v>
       </c>
-      <c r="C31" t="s">
-        <v>249</v>
-      </c>
       <c r="D31" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="7">
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C32" t="s">
         <v>250</v>
       </c>
-      <c r="C32" t="s">
-        <v>251</v>
-      </c>
       <c r="D32" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="7">
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C33" t="s">
         <v>252</v>
       </c>
-      <c r="C33" t="s">
-        <v>253</v>
-      </c>
       <c r="D33" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4086,408 +4143,408 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O126"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="42.6328125" customWidth="1"/>
-    <col min="2" max="2" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.6640625" customWidth="1"/>
+    <col min="2" max="2" width="35.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" style="7" customWidth="1"/>
-    <col min="4" max="4" width="38.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="80.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="80.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
+        <v>361</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>362</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>363</v>
+      </c>
+      <c r="F1" t="s">
+        <v>141</v>
+      </c>
+      <c r="G1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H1" t="s">
+        <v>143</v>
+      </c>
+      <c r="I1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J1" t="s">
+        <v>145</v>
+      </c>
+      <c r="K1" t="s">
+        <v>146</v>
+      </c>
+      <c r="L1" t="s">
+        <v>147</v>
+      </c>
+      <c r="M1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N1" t="s">
+        <v>149</v>
+      </c>
+      <c r="O1" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
+      <c r="A2" s="31" t="s">
+        <v>364</v>
+      </c>
+      <c r="B2" s="28" t="s">
         <v>365</v>
-      </c>
-      <c r="B1" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="C1" s="33" t="s">
-        <v>366</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>367</v>
-      </c>
-      <c r="F1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G1" t="s">
-        <v>143</v>
-      </c>
-      <c r="H1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I1" t="s">
-        <v>145</v>
-      </c>
-      <c r="J1" t="s">
-        <v>146</v>
-      </c>
-      <c r="K1" t="s">
-        <v>147</v>
-      </c>
-      <c r="L1" t="s">
-        <v>148</v>
-      </c>
-      <c r="M1" t="s">
-        <v>149</v>
-      </c>
-      <c r="N1" t="s">
-        <v>150</v>
-      </c>
-      <c r="O1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="31" t="s">
-        <v>368</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>369</v>
       </c>
       <c r="C2" s="34">
         <v>28</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="C3" s="34">
         <v>1</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" s="35">
         <v>2</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C5" s="35">
         <v>2</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C6" s="35">
         <v>2</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C7" s="34">
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" ht="29" x14ac:dyDescent="0.35">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C8" s="35">
         <v>24</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C9" s="35">
         <v>4</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C10" s="35">
         <v>1</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C11" s="34">
         <v>3</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C12" s="34">
         <v>1</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C13" s="35">
         <v>1</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C14" s="34">
         <v>2</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C15" s="35">
         <v>16</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C16" s="34">
         <v>2</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="C17" s="34">
+        <v>1</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>191</v>
       </c>
-      <c r="B17" s="28" t="s">
-        <v>193</v>
-      </c>
-      <c r="C17" s="34">
-        <v>1</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="C18" s="34">
+        <v>1</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>371</v>
+      </c>
+      <c r="C19" s="35">
+        <v>1</v>
+      </c>
+      <c r="D19" s="30" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="C20" s="34">
+        <v>1</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="B21" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="34">
+        <v>1</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="29" t="s">
+        <v>170</v>
+      </c>
+      <c r="B22" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="C22" s="35">
+        <v>1</v>
+      </c>
+      <c r="D22" s="30" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="C18" s="34">
-        <v>1</v>
-      </c>
-      <c r="D18" s="28" t="s">
+      <c r="B23" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="C23" s="34">
+        <v>1</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="27" t="s">
+        <v>374</v>
+      </c>
+      <c r="B24" s="28" t="s">
+        <v>160</v>
+      </c>
+      <c r="C24" s="34">
+        <v>1</v>
+      </c>
+      <c r="D24" s="28" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="C25" s="34">
+        <v>1</v>
+      </c>
+      <c r="D25" s="28" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="29" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>375</v>
-      </c>
-      <c r="C19" s="35">
-        <v>1</v>
-      </c>
-      <c r="D19" s="30" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="C20" s="34">
-        <v>1</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="B21" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="C21" s="34">
-        <v>1</v>
-      </c>
-      <c r="D21" s="28" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="29" t="s">
-        <v>171</v>
-      </c>
-      <c r="B22" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="C22" s="35">
-        <v>1</v>
-      </c>
-      <c r="D22" s="30" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>166</v>
-      </c>
-      <c r="C23" s="34">
-        <v>1</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="27" t="s">
-        <v>378</v>
-      </c>
-      <c r="B24" s="28" t="s">
-        <v>161</v>
-      </c>
-      <c r="C24" s="34">
-        <v>1</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>168</v>
-      </c>
-      <c r="C25" s="34">
-        <v>1</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>73</v>
@@ -4496,113 +4553,113 @@
         <v>1</v>
       </c>
       <c r="D26" s="28" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="C27" s="35">
+        <v>1</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="29" t="s">
+        <v>379</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="35">
+        <v>1</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="29" t="s">
+        <v>380</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>381</v>
+      </c>
+      <c r="C29" s="35">
+        <v>1</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="29" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="29" t="s">
-        <v>189</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="35">
-        <v>1</v>
-      </c>
-      <c r="D27" s="30" t="s">
+      <c r="B30" s="30" t="s">
+        <v>383</v>
+      </c>
+      <c r="C30" s="35">
+        <v>1</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="C31" s="34">
+        <v>1</v>
+      </c>
+      <c r="D31" s="28" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="29" t="s">
-        <v>383</v>
-      </c>
-      <c r="B28" s="30" t="s">
-        <v>155</v>
-      </c>
-      <c r="C28" s="35">
-        <v>1</v>
-      </c>
-      <c r="D28" s="30" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="29" t="s">
-        <v>384</v>
-      </c>
-      <c r="B29" s="30" t="s">
-        <v>385</v>
-      </c>
-      <c r="C29" s="35">
-        <v>1</v>
-      </c>
-      <c r="D29" s="30" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="29" t="s">
-        <v>386</v>
-      </c>
-      <c r="B30" s="30" t="s">
-        <v>387</v>
-      </c>
-      <c r="C30" s="35">
-        <v>1</v>
-      </c>
-      <c r="D30" s="30" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="27" t="s">
-        <v>179</v>
-      </c>
-      <c r="B31" s="28" t="s">
-        <v>180</v>
-      </c>
-      <c r="C31" s="34">
-        <v>1</v>
-      </c>
-      <c r="D31" s="28" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="29" t="s">
+        <v>193</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="C32" s="35">
+        <v>1</v>
+      </c>
+      <c r="D32" s="30" t="s">
         <v>194</v>
       </c>
-      <c r="B32" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="C32" s="35">
-        <v>1</v>
-      </c>
-      <c r="D32" s="30" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="78" spans="6:13" x14ac:dyDescent="0.35">
+    </row>
+    <row r="78" spans="6:13" x14ac:dyDescent="0.2">
       <c r="G78" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H78">
         <v>1296592</v>
       </c>
       <c r="I78" t="s">
+        <v>174</v>
+      </c>
+      <c r="J78" t="s">
         <v>175</v>
-      </c>
-      <c r="J78" t="s">
-        <v>176</v>
       </c>
       <c r="M78" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="79" spans="6:13" x14ac:dyDescent="0.35">
+    <row r="79" spans="6:13" x14ac:dyDescent="0.2">
       <c r="F79" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G79" t="s">
         <v>73</v>
@@ -4611,17 +4668,17 @@
         <v>1462926</v>
       </c>
       <c r="I79" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="81" spans="11:11" x14ac:dyDescent="0.35">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="81" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K81" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="126" spans="14:14" x14ac:dyDescent="0.35">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="126" spans="14:14" x14ac:dyDescent="0.2">
       <c r="N126" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update p-channel mosfet from BSH203 to SSM3J328R
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wmedu-my.sharepoint.com/personal/joslater_wm_edu/Documents/VIMS/aubrey_project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{AB5E46A4-20F2-224B-A54B-BAAB896D7AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1DC8607-A9B0-004D-BB5D-A2F480AC0CD8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70E16C9-B35C-B548-8867-DB17C62CBEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="440">
   <si>
     <t>Part Description</t>
   </si>
@@ -372,15 +372,9 @@
     <t>MCP1700T-3002E/TT</t>
   </si>
   <si>
-    <t>Mosfet P-FET SOT23-3 BH203,215</t>
-  </si>
-  <si>
     <t>miller.lbr\MOSFET-PCHANNEL</t>
   </si>
   <si>
-    <t>Nexperia</t>
-  </si>
-  <si>
     <t>BSH203,215</t>
   </si>
   <si>
@@ -402,9 +396,6 @@
     <t>miller.lbr\MICROSD_MOLEX_REVERSECURRENT</t>
   </si>
   <si>
-    <t>WM24066CT-ND</t>
-  </si>
-  <si>
     <t>MicroSD card slot push-push</t>
   </si>
   <si>
@@ -1375,9 +1366,6 @@
   </si>
   <si>
     <t>311-3486-2-ND</t>
-  </si>
-  <si>
-    <t>FIND SUBSTITUTE</t>
   </si>
   <si>
     <t>slater substitute</t>
@@ -1408,10 +1396,25 @@
     <t>FIND SUBSTITUTE, OR AVAILABLE AT https://www.lcsc.com/product-detail/C131334.html</t>
   </si>
   <si>
-    <t>USE ALT</t>
-  </si>
-  <si>
     <t>NEED SUB IF USING DIFF HEADER</t>
+  </si>
+  <si>
+    <t>GCT</t>
+  </si>
+  <si>
+    <t>MEM2052-00-195-00-A</t>
+  </si>
+  <si>
+    <t>2073-MEM2052-00-195-00-ACT-ND</t>
+  </si>
+  <si>
+    <t>slater substitute alt for main</t>
+  </si>
+  <si>
+    <t>Toshiba</t>
+  </si>
+  <si>
+    <t>P-Channel 20 V 6A (Ta) 1W (Ta) Surface Mount SOT-23F</t>
   </si>
 </sst>
 </file>
@@ -1506,10 +1509,8 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1585,7 +1586,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1664,14 +1665,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2055,7 +2052,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="15" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -2084,19 +2081,19 @@
         <v>12</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="K2" s="15" t="s">
+        <v>342</v>
+      </c>
+      <c r="L2" s="15" t="s">
         <v>345</v>
       </c>
-      <c r="L2" s="15" t="s">
-        <v>348</v>
-      </c>
       <c r="M2" s="15" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
@@ -2155,7 +2152,7 @@
     </row>
     <row r="5" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -2164,13 +2161,13 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E5" s="7">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="G5" s="6">
         <v>0.73</v>
@@ -2181,8 +2178,8 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="43" t="s">
-        <v>291</v>
+      <c r="A6" s="40" t="s">
+        <v>288</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -2191,13 +2188,13 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="E6" s="7">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="G6" s="6">
         <v>0.65</v>
@@ -2207,7 +2204,7 @@
         <v>0.65</v>
       </c>
       <c r="I6" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2239,7 +2236,7 @@
     </row>
     <row r="8" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
@@ -2248,13 +2245,13 @@
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E8" s="7">
         <v>2</v>
       </c>
       <c r="F8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G8" s="6">
         <v>0.1</v>
@@ -2401,22 +2398,22 @@
     </row>
     <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D14" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E14" s="7">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="G14" s="6">
         <v>0.62</v>
@@ -2426,16 +2423,16 @@
         <v>0.62</v>
       </c>
       <c r="J14" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="K14" t="s">
+        <v>344</v>
+      </c>
+      <c r="L14" t="s">
+        <v>348</v>
+      </c>
+      <c r="M14" t="s">
         <v>347</v>
-      </c>
-      <c r="L14" t="s">
-        <v>351</v>
-      </c>
-      <c r="M14" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2467,7 +2464,7 @@
     </row>
     <row r="16" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B16" t="s">
         <v>46</v>
@@ -2476,13 +2473,13 @@
         <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E16" s="7">
         <v>16</v>
       </c>
       <c r="F16" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="G16" s="6">
         <v>1.22</v>
@@ -2494,19 +2491,19 @@
     </row>
     <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E17" s="7">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="G17" s="6">
         <v>12.46</v>
@@ -2516,10 +2513,10 @@
         <v>12.46</v>
       </c>
       <c r="J17" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="K17" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2557,13 +2554,13 @@
         <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E19" s="7">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="G19" s="6">
         <v>1.03</v>
@@ -2600,7 +2597,7 @@
         <v>3.84</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2627,7 +2624,7 @@
         <v>1.6</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2655,10 +2652,10 @@
       </c>
       <c r="I22" s="39"/>
       <c r="J22" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="K22" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2768,7 +2765,7 @@
     </row>
     <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B27" t="s">
         <v>92</v>
@@ -2793,30 +2790,30 @@
         <v>0.51</v>
       </c>
       <c r="J27" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K27" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="40" t="s">
+        <v>439</v>
+      </c>
+      <c r="B28" t="s">
         <v>95</v>
       </c>
-      <c r="B28" t="s">
-        <v>96</v>
-      </c>
       <c r="C28" t="s">
-        <v>97</v>
+        <v>438</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>349</v>
       </c>
       <c r="E28" s="7">
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>99</v>
+        <v>350</v>
       </c>
       <c r="G28" s="6">
         <v>0.38</v>
@@ -2825,34 +2822,34 @@
         <f t="shared" si="0"/>
         <v>0.38</v>
       </c>
-      <c r="I28" s="40" t="s">
+      <c r="I28" s="41" t="s">
         <v>437</v>
       </c>
       <c r="J28" t="s">
-        <v>352</v>
+        <v>96</v>
       </c>
       <c r="K28" t="s">
-        <v>353</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B29" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" t="s">
         <v>101</v>
       </c>
-      <c r="B29" t="s">
-        <v>102</v>
-      </c>
-      <c r="C29" t="s">
-        <v>103</v>
-      </c>
       <c r="D29" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E29" s="7">
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="G29" s="6">
         <v>0.72</v>
@@ -2863,50 +2860,50 @@
       </c>
     </row>
     <row r="30" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="4" t="s">
-        <v>106</v>
+      <c r="A30" s="40" t="s">
+        <v>103</v>
       </c>
       <c r="B30" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C30" t="s">
-        <v>72</v>
-      </c>
-      <c r="D30">
-        <v>5027740891</v>
+        <v>434</v>
+      </c>
+      <c r="D30" t="s">
+        <v>435</v>
       </c>
       <c r="E30" s="7">
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>105</v>
+        <v>436</v>
       </c>
       <c r="G30" s="6">
-        <v>3.64</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="H30" s="6">
         <f t="shared" si="0"/>
-        <v>3.64</v>
-      </c>
-      <c r="I30" s="39" t="s">
-        <v>430</v>
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="I30" s="41" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>433</v>
-      </c>
-      <c r="C31" s="41" t="s">
-        <v>103</v>
-      </c>
-      <c r="D31" s="41" t="s">
-        <v>434</v>
-      </c>
-      <c r="E31" s="42">
-        <v>1</v>
-      </c>
-      <c r="F31" s="41" t="s">
-        <v>435</v>
+        <v>429</v>
+      </c>
+      <c r="C31" t="s">
+        <v>101</v>
+      </c>
+      <c r="D31" t="s">
+        <v>430</v>
+      </c>
+      <c r="E31" s="7">
+        <v>1</v>
+      </c>
+      <c r="F31" t="s">
+        <v>431</v>
       </c>
       <c r="G31" s="6">
         <v>1.25</v>
@@ -2915,28 +2912,28 @@
         <f t="shared" si="0"/>
         <v>1.25</v>
       </c>
-      <c r="I31" s="41" t="s">
-        <v>431</v>
+      <c r="I31" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C32" t="s">
         <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="E32" s="7">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="G32" s="6">
         <v>2.74</v>
@@ -2946,18 +2943,18 @@
         <v>2.74</v>
       </c>
       <c r="J32" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="K32" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D33">
         <v>8195</v>
@@ -2966,7 +2963,7 @@
         <v>16</v>
       </c>
       <c r="F33" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G33" s="6">
         <v>0.18</v>
@@ -2978,22 +2975,22 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B34" t="s">
+        <v>125</v>
+      </c>
+      <c r="C34" t="s">
+        <v>126</v>
+      </c>
+      <c r="D34" t="s">
+        <v>127</v>
+      </c>
+      <c r="E34" s="7">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
         <v>128</v>
-      </c>
-      <c r="C34" t="s">
-        <v>129</v>
-      </c>
-      <c r="D34" t="s">
-        <v>130</v>
-      </c>
-      <c r="E34" s="7">
-        <v>1</v>
-      </c>
-      <c r="F34" t="s">
-        <v>131</v>
       </c>
       <c r="G34" s="6">
         <v>0.75</v>
@@ -3005,19 +3002,19 @@
     </row>
     <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C35" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D35" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E35" s="7">
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="G35" s="6">
         <v>1.71</v>
@@ -3029,22 +3026,22 @@
     </row>
     <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B36" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C36" t="s">
         <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E36" s="7">
         <v>1</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="G36" s="6">
         <v>0.64</v>
@@ -3056,19 +3053,19 @@
     </row>
     <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B37" t="s">
+        <v>285</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>286</v>
+      </c>
+      <c r="E37" s="7">
+        <v>1</v>
+      </c>
+      <c r="F37" s="21" t="s">
         <v>287</v>
-      </c>
-      <c r="B37" t="s">
-        <v>288</v>
-      </c>
-      <c r="D37" s="21" t="s">
-        <v>289</v>
-      </c>
-      <c r="E37" s="7">
-        <v>1</v>
-      </c>
-      <c r="F37" s="21" t="s">
-        <v>290</v>
       </c>
       <c r="G37" s="6">
         <v>0.67</v>
@@ -3105,7 +3102,7 @@
         <v>0.16</v>
       </c>
       <c r="I38" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3132,7 +3129,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="I39" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3159,7 +3156,7 @@
         <v>1.5</v>
       </c>
       <c r="I40" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
@@ -3168,42 +3165,42 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G42" s="19" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="H42" s="19">
         <f>SUM(H3:H37)</f>
-        <v>72.669999999999973</v>
+        <v>70.149999999999977</v>
       </c>
       <c r="I42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C44" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D44" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F44" t="s">
+        <v>294</v>
+      </c>
+      <c r="G44" s="6" t="s">
         <v>297</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>300</v>
       </c>
       <c r="H44" s="12">
         <v>4.62</v>
       </c>
       <c r="I44" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
@@ -3212,15 +3209,15 @@
     <row r="54" spans="1:11" ht="30.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="56" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E57" s="7">
         <v>1</v>
@@ -3233,15 +3230,15 @@
         <v>15.066666666666668</v>
       </c>
       <c r="I57" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="E58" s="7">
         <v>16</v>
@@ -3262,16 +3259,16 @@
     </row>
     <row r="60" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G60" s="11"/>
     </row>
     <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C61" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E61" s="7">
         <v>1</v>
@@ -3284,15 +3281,15 @@
         <v>0</v>
       </c>
       <c r="I61" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="C62" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E62" s="7">
         <v>1</v>
@@ -3305,22 +3302,22 @@
     </row>
     <row r="64" spans="1:11" ht="20" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E64"/>
       <c r="F64" s="9" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="E65" s="7">
         <v>1</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="G65" s="6">
         <v>9.99</v>
@@ -3332,13 +3329,13 @@
     </row>
     <row r="66" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E66" s="7">
         <v>1</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G66" s="6">
         <v>6.99</v>
@@ -3356,28 +3353,28 @@
       <c r="A68"/>
       <c r="E68"/>
       <c r="G68" s="19" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>117.33666666666667</v>
+        <v>114.81666666666668</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E69"/>
     </row>
     <row r="70" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E70" s="7">
         <v>1</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G70" s="6">
         <v>44.22</v>
@@ -3387,47 +3384,47 @@
         <v>0</v>
       </c>
       <c r="I70" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C71" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="D71" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E71" s="7">
         <v>1</v>
       </c>
       <c r="F71" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="G71" s="6">
         <v>64.5</v>
       </c>
       <c r="I71" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C72" t="s">
+        <v>338</v>
+      </c>
+      <c r="D72" t="s">
+        <v>339</v>
+      </c>
+      <c r="E72" s="7">
+        <v>1</v>
+      </c>
+      <c r="F72" t="s">
         <v>332</v>
-      </c>
-      <c r="C72" t="s">
-        <v>341</v>
-      </c>
-      <c r="D72" t="s">
-        <v>342</v>
-      </c>
-      <c r="E72" s="7">
-        <v>1</v>
-      </c>
-      <c r="F72" t="s">
-        <v>335</v>
       </c>
       <c r="G72" s="6">
         <v>129.94999999999999</v>
@@ -3435,19 +3432,19 @@
     </row>
     <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C73" t="s">
+        <v>338</v>
+      </c>
+      <c r="D73" t="s">
+        <v>340</v>
+      </c>
+      <c r="E73" s="7">
+        <v>1</v>
+      </c>
+      <c r="F73" s="24" t="s">
         <v>333</v>
-      </c>
-      <c r="C73" t="s">
-        <v>341</v>
-      </c>
-      <c r="D73" t="s">
-        <v>343</v>
-      </c>
-      <c r="E73" s="7">
-        <v>1</v>
-      </c>
-      <c r="F73" s="24" t="s">
-        <v>336</v>
       </c>
       <c r="G73" s="6">
         <v>129</v>
@@ -3458,25 +3455,25 @@
     </row>
     <row r="76" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" s="10" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="H76" s="12"/>
     </row>
     <row r="77" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C77" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D77" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E77" s="7">
         <v>16</v>
       </c>
       <c r="F77" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="G77" s="6">
         <v>1.31</v>
@@ -3488,19 +3485,19 @@
     </row>
     <row r="78" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C78" t="s">
+        <v>298</v>
+      </c>
+      <c r="D78" t="s">
+        <v>300</v>
+      </c>
+      <c r="E78" s="7">
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
         <v>301</v>
-      </c>
-      <c r="D78" t="s">
-        <v>303</v>
-      </c>
-      <c r="E78" s="7">
-        <v>1</v>
-      </c>
-      <c r="F78" t="s">
-        <v>304</v>
       </c>
       <c r="G78" s="6">
         <v>18.28</v>
@@ -3512,19 +3509,19 @@
     </row>
     <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="C79" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D79" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E79" s="7">
         <v>1</v>
       </c>
       <c r="F79" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="G79" s="6">
         <v>10.81</v>
@@ -3536,19 +3533,19 @@
     </row>
     <row r="80" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C80" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D80" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E80" s="7">
         <v>1</v>
       </c>
       <c r="F80" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="G80" s="6">
         <v>7.8</v>
@@ -3560,36 +3557,36 @@
     </row>
     <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="C81" t="s">
         <v>422</v>
       </c>
-      <c r="C81" t="s">
-        <v>425</v>
-      </c>
       <c r="D81" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="E81">
         <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C82" t="s">
+        <v>320</v>
+      </c>
+      <c r="D82" t="s">
+        <v>321</v>
+      </c>
+      <c r="E82" s="7">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
         <v>322</v>
-      </c>
-      <c r="C82" t="s">
-        <v>323</v>
-      </c>
-      <c r="D82" t="s">
-        <v>324</v>
-      </c>
-      <c r="E82" s="7">
-        <v>1</v>
-      </c>
-      <c r="F82" t="s">
-        <v>325</v>
       </c>
       <c r="G82" s="6">
         <v>2.19</v>
@@ -3601,19 +3598,19 @@
     </row>
     <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C83" t="s">
+        <v>312</v>
+      </c>
+      <c r="D83" t="s">
+        <v>313</v>
+      </c>
+      <c r="E83" s="7">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
         <v>314</v>
-      </c>
-      <c r="C83" t="s">
-        <v>315</v>
-      </c>
-      <c r="D83" t="s">
-        <v>316</v>
-      </c>
-      <c r="E83" s="7">
-        <v>1</v>
-      </c>
-      <c r="F83" t="s">
-        <v>317</v>
       </c>
       <c r="G83" s="6">
         <v>3.51</v>
@@ -3625,13 +3622,13 @@
     </row>
     <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C84" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D84" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="E84" s="7">
         <v>16</v>
@@ -3674,16 +3671,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>194</v>
+      </c>
+      <c r="C1" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>199</v>
-      </c>
       <c r="D1" s="15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -3691,13 +3688,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -3705,13 +3702,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D3" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -3719,13 +3716,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D4" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -3733,13 +3730,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C5" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -3747,13 +3744,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C6" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="D6" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -3761,13 +3758,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -3775,13 +3772,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C8" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D8" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -3789,13 +3786,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C9" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D9" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -3803,13 +3800,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C10" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D10" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -3817,13 +3814,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C11" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D11" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -3831,13 +3828,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C12" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D12" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -3845,13 +3842,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C13" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D13" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -3859,13 +3856,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C14" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D14" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -3873,13 +3870,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="D15" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -3887,13 +3884,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C16" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D16" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -3901,13 +3898,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C17" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D17" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -3915,13 +3912,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C18" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D18" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -3929,13 +3926,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D19" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -3943,13 +3940,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C20" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D20" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -3957,13 +3954,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C21" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D21" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -3971,13 +3968,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C22" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D22" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -3985,13 +3982,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C23" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D23" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -3999,13 +3996,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C24" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D24" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -4013,13 +4010,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C25" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D25" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -4027,13 +4024,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C26" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D26" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4041,13 +4038,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C27" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D27" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -4055,13 +4052,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C28" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D28" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -4069,13 +4066,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C29" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D29" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -4083,13 +4080,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C30" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D30" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -4097,13 +4094,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C31" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D31" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -4111,13 +4108,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C32" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D32" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -4125,13 +4122,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C33" t="s">
+        <v>249</v>
+      </c>
+      <c r="D33" t="s">
         <v>251</v>
-      </c>
-      <c r="C33" t="s">
-        <v>252</v>
-      </c>
-      <c r="D33" t="s">
-        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4164,387 +4161,387 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B1" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="33" t="s">
+        <v>359</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>360</v>
+      </c>
+      <c r="F1" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" t="s">
         <v>139</v>
       </c>
-      <c r="C1" s="33" t="s">
-        <v>362</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>363</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" t="s">
         <v>141</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>142</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>143</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>144</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>145</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>146</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>147</v>
-      </c>
-      <c r="M1" t="s">
-        <v>148</v>
-      </c>
-      <c r="N1" t="s">
-        <v>149</v>
-      </c>
-      <c r="O1" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C2" s="34">
         <v>28</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C3" s="34">
         <v>1</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B4" s="30" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C4" s="35">
         <v>2</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C5" s="35">
         <v>2</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B6" s="30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C6" s="35">
         <v>2</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C7" s="34">
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C8" s="35">
         <v>24</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C9" s="35">
         <v>4</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C10" s="35">
         <v>1</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C11" s="34">
         <v>3</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C12" s="34">
         <v>1</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="29" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B13" s="30" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C13" s="35">
         <v>1</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C14" s="34">
         <v>2</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B15" s="30" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C15" s="35">
         <v>16</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C16" s="34">
         <v>2</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="27" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C17" s="34">
         <v>1</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B18" s="28" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C18" s="34">
         <v>1</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="29" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C19" s="35">
         <v>1</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="27" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C20" s="34">
         <v>1</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C21" s="34">
         <v>1</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="29" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C22" s="35">
         <v>1</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="27" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B23" s="28" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C23" s="34">
         <v>1</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B24" s="28" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C24" s="34">
         <v>1</v>
       </c>
       <c r="D24" s="28" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="27" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C25" s="34">
         <v>1</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>73</v>
@@ -4553,105 +4550,105 @@
         <v>1</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="29" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C27" s="35">
         <v>1</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="29" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C28" s="35">
         <v>1</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="29" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C29" s="35">
         <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="29" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B30" s="30" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C30" s="35">
         <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="27" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B31" s="28" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C31" s="34">
         <v>1</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="29" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B32" s="30" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C32" s="35">
         <v>1</v>
       </c>
       <c r="D32" s="30" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" spans="6:13" x14ac:dyDescent="0.2">
       <c r="G78" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="H78">
         <v>1296592</v>
       </c>
       <c r="I78" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="J78" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="M78" t="s">
         <v>93</v>
@@ -4659,7 +4656,7 @@
     </row>
     <row r="79" spans="6:13" x14ac:dyDescent="0.2">
       <c r="F79" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G79" t="s">
         <v>73</v>
@@ -4668,17 +4665,17 @@
         <v>1462926</v>
       </c>
       <c r="I79" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="81" spans="11:11" x14ac:dyDescent="0.2">
       <c r="K81" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="126" spans="14:14" x14ac:dyDescent="0.2">
       <c r="N126" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Moved changes to Rev I and fixed DRC errors
Made new copy of KiCad project in Rev I and fixed some electric rules checker errors and warnings and some design rules checker errors and warnings
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70E16C9-B35C-B548-8867-DB17C62CBEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0643BE-2144-E445-A38C-3DA5758A2B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2816,11 +2816,11 @@
         <v>350</v>
       </c>
       <c r="G28" s="6">
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="H28" s="6">
         <f t="shared" si="0"/>
-        <v>0.38</v>
+        <v>0.42</v>
       </c>
       <c r="I28" s="41" t="s">
         <v>437</v>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="H42" s="19">
         <f>SUM(H3:H37)</f>
-        <v>70.149999999999977</v>
+        <v>70.189999999999984</v>
       </c>
       <c r="I42" t="s">
         <v>121</v>
@@ -3357,7 +3357,7 @@
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>114.81666666666668</v>
+        <v>114.85666666666668</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated parts list with cable sub
</commit_message>
<xml_diff>
--- a/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
+++ b/KiCad_files/MusselGapeTracker_RevH/MusselGapeTracker_RevH_parts_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jack/Documents/GitHub/MusselGapeTracker_hardware/KiCad_files/MusselGapeTracker_RevH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0643BE-2144-E445-A38C-3DA5758A2B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B149A335-57B5-464C-8AFD-EC4F145D2DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="441">
   <si>
     <t>Part Description</t>
   </si>
@@ -969,18 +969,9 @@
     <t>Cable Feedthrough 2.5mm-6.5mm Polyamide PG7 Black</t>
   </si>
   <si>
-    <t>CN230-B-100-ND</t>
-  </si>
-  <si>
-    <t>2725-2828-BL-01000-A</t>
-  </si>
-  <si>
     <t>CNC Tech</t>
   </si>
   <si>
-    <t>$0.26/ft</t>
-  </si>
-  <si>
     <t>Serpac</t>
   </si>
   <si>
@@ -1369,6 +1360,51 @@
   </si>
   <si>
     <t>slater substitute</t>
+  </si>
+  <si>
+    <t>CD74HC4067PWR multiplexer 16 channel (24-TSSOP 4.4x7.8mm, 0.65mm pitch)</t>
+  </si>
+  <si>
+    <t>CD74HC4067PWR</t>
+  </si>
+  <si>
+    <t>296-CD74HC4067PWRCT-ND</t>
+  </si>
+  <si>
+    <t>FIND SUBSTITUTE, OR AVAILABLE AT https://www.lcsc.com/product-detail/C131334.html</t>
+  </si>
+  <si>
+    <t>NEED SUB IF USING DIFF HEADER</t>
+  </si>
+  <si>
+    <t>GCT</t>
+  </si>
+  <si>
+    <t>MEM2052-00-195-00-A</t>
+  </si>
+  <si>
+    <t>2073-MEM2052-00-195-00-ACT-ND</t>
+  </si>
+  <si>
+    <t>slater substitute alt for main</t>
+  </si>
+  <si>
+    <t>Toshiba</t>
+  </si>
+  <si>
+    <t>P-Channel 20 V 6A (Ta) 1W (Ta) Surface Mount SOT-23F</t>
+  </si>
+  <si>
+    <t>^/ft</t>
+  </si>
+  <si>
+    <t>^ft</t>
+  </si>
+  <si>
+    <t>CN306-100-ND</t>
+  </si>
+  <si>
+    <t>2725-2828-BE-01000-A</t>
   </si>
   <si>
     <r>
@@ -1377,44 +1413,11 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color rgb="FFFF0000"/>
+        <color theme="1"/>
         <rFont val="Calibri (Body)"/>
       </rPr>
-      <t>FIND SUBSTITUTE</t>
+      <t>slater substitute</t>
     </r>
-  </si>
-  <si>
-    <t>CD74HC4067PWR multiplexer 16 channel (24-TSSOP 4.4x7.8mm, 0.65mm pitch)</t>
-  </si>
-  <si>
-    <t>CD74HC4067PWR</t>
-  </si>
-  <si>
-    <t>296-CD74HC4067PWRCT-ND</t>
-  </si>
-  <si>
-    <t>FIND SUBSTITUTE, OR AVAILABLE AT https://www.lcsc.com/product-detail/C131334.html</t>
-  </si>
-  <si>
-    <t>NEED SUB IF USING DIFF HEADER</t>
-  </si>
-  <si>
-    <t>GCT</t>
-  </si>
-  <si>
-    <t>MEM2052-00-195-00-A</t>
-  </si>
-  <si>
-    <t>2073-MEM2052-00-195-00-ACT-ND</t>
-  </si>
-  <si>
-    <t>slater substitute alt for main</t>
-  </si>
-  <si>
-    <t>Toshiba</t>
-  </si>
-  <si>
-    <t>P-Channel 20 V 6A (Ta) 1W (Ta) Surface Mount SOT-23F</t>
   </si>
 </sst>
 </file>
@@ -1586,7 +1589,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1669,6 +1672,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2052,7 +2056,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="15" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -2081,19 +2085,19 @@
         <v>12</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="K2" s="15" t="s">
+        <v>339</v>
+      </c>
+      <c r="L2" s="15" t="s">
         <v>342</v>
       </c>
-      <c r="L2" s="15" t="s">
-        <v>345</v>
-      </c>
       <c r="M2" s="15" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="32" x14ac:dyDescent="0.2">
@@ -2188,13 +2192,13 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="E6" s="7">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="G6" s="6">
         <v>0.65</v>
@@ -2204,7 +2208,7 @@
         <v>0.65</v>
       </c>
       <c r="I6" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2398,22 +2402,22 @@
     </row>
     <row r="14" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B14" t="s">
         <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="D14" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="E14" s="7">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G14" s="6">
         <v>0.62</v>
@@ -2423,16 +2427,16 @@
         <v>0.62</v>
       </c>
       <c r="J14" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="K14" t="s">
+        <v>341</v>
+      </c>
+      <c r="L14" t="s">
+        <v>345</v>
+      </c>
+      <c r="M14" t="s">
         <v>344</v>
-      </c>
-      <c r="L14" t="s">
-        <v>348</v>
-      </c>
-      <c r="M14" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="16" x14ac:dyDescent="0.2">
@@ -2491,19 +2495,19 @@
     </row>
     <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="C17" t="s">
         <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E17" s="7">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="G17" s="6">
         <v>12.46</v>
@@ -2513,10 +2517,10 @@
         <v>12.46</v>
       </c>
       <c r="J17" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="K17" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -2597,7 +2601,7 @@
         <v>3.84</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2624,7 +2628,7 @@
         <v>1.6</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2652,10 +2656,10 @@
       </c>
       <c r="I22" s="39"/>
       <c r="J22" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="K22" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -2765,7 +2769,7 @@
     </row>
     <row r="27" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="B27" t="s">
         <v>92</v>
@@ -2793,27 +2797,27 @@
         <v>169</v>
       </c>
       <c r="K27" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="40" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="B28" t="s">
         <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="D28" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E28" s="7">
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="G28" s="6">
         <v>0.42</v>
@@ -2823,7 +2827,7 @@
         <v>0.42</v>
       </c>
       <c r="I28" s="41" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="J28" t="s">
         <v>96</v>
@@ -2849,7 +2853,7 @@
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="G29" s="6">
         <v>0.72</v>
@@ -2867,16 +2871,16 @@
         <v>102</v>
       </c>
       <c r="C30" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="D30" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="E30" s="7">
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="G30" s="6">
         <v>1.1200000000000001</v>
@@ -2886,24 +2890,24 @@
         <v>1.1200000000000001</v>
       </c>
       <c r="I30" s="41" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="37" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="C31" t="s">
         <v>101</v>
       </c>
       <c r="D31" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="E31" s="7">
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="G31" s="6">
         <v>1.25</v>
@@ -2913,7 +2917,7 @@
         <v>1.25</v>
       </c>
       <c r="I31" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="16" x14ac:dyDescent="0.2">
@@ -2927,13 +2931,13 @@
         <v>93</v>
       </c>
       <c r="D32" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E32" s="7">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="G32" s="6">
         <v>2.74</v>
@@ -2943,10 +2947,10 @@
         <v>2.74</v>
       </c>
       <c r="J32" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="K32" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -2975,7 +2979,7 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="B34" t="s">
         <v>125</v>
@@ -3002,19 +3006,19 @@
     </row>
     <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C35" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D35" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E35" s="7">
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="G35" s="6">
         <v>1.71</v>
@@ -3102,7 +3106,7 @@
         <v>0.16</v>
       </c>
       <c r="I38" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3129,7 +3133,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="I39" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -3156,7 +3160,7 @@
         <v>1.5</v>
       </c>
       <c r="I40" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
@@ -3181,29 +3185,39 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="40" t="s">
         <v>110</v>
       </c>
       <c r="C44" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D44" t="s">
-        <v>295</v>
+        <v>439</v>
+      </c>
+      <c r="E44" s="7">
+        <v>72</v>
       </c>
       <c r="F44" t="s">
-        <v>294</v>
-      </c>
-      <c r="G44" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="H44" s="12">
-        <v>4.62</v>
+        <v>438</v>
+      </c>
+      <c r="G44" s="12">
+        <v>0.26</v>
+      </c>
+      <c r="H44" s="42">
+        <f>E44*G44</f>
+        <v>18.72</v>
       </c>
       <c r="I44" t="s">
-        <v>428</v>
+        <v>440</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E45" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>436</v>
+      </c>
       <c r="H45" s="12"/>
     </row>
     <row r="54" spans="1:11" ht="30.5" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3214,10 +3228,10 @@
     </row>
     <row r="57" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="E57" s="7">
         <v>1</v>
@@ -3235,10 +3249,10 @@
     </row>
     <row r="58" spans="1:11" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="E58" s="7">
         <v>16</v>
@@ -3265,10 +3279,10 @@
     </row>
     <row r="61" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="C61" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E61" s="7">
         <v>1</v>
@@ -3286,10 +3300,10 @@
     </row>
     <row r="62" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="C62" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E62" s="7">
         <v>1</v>
@@ -3306,18 +3320,18 @@
       </c>
       <c r="E64"/>
       <c r="F64" s="9" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="E65" s="7">
         <v>1</v>
       </c>
       <c r="F65" s="36" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="G65" s="6">
         <v>9.99</v>
@@ -3353,16 +3367,16 @@
       <c r="A68"/>
       <c r="E68"/>
       <c r="G68" s="19" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="H68" s="12">
         <f>SUM(H44:H66,H3:H37)</f>
-        <v>114.85666666666668</v>
+        <v>128.95666666666665</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E69"/>
     </row>
@@ -3389,19 +3403,19 @@
     </row>
     <row r="71" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C71" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D71" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E71" s="7">
         <v>1</v>
       </c>
       <c r="F71" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="G71" s="6">
         <v>64.5</v>
@@ -3412,19 +3426,19 @@
     </row>
     <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C72" t="s">
+        <v>335</v>
+      </c>
+      <c r="D72" t="s">
+        <v>336</v>
+      </c>
+      <c r="E72" s="7">
+        <v>1</v>
+      </c>
+      <c r="F72" t="s">
         <v>329</v>
-      </c>
-      <c r="C72" t="s">
-        <v>338</v>
-      </c>
-      <c r="D72" t="s">
-        <v>339</v>
-      </c>
-      <c r="E72" s="7">
-        <v>1</v>
-      </c>
-      <c r="F72" t="s">
-        <v>332</v>
       </c>
       <c r="G72" s="6">
         <v>129.94999999999999</v>
@@ -3432,19 +3446,19 @@
     </row>
     <row r="73" spans="1:9" ht="17" x14ac:dyDescent="0.25">
       <c r="A73" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C73" t="s">
+        <v>335</v>
+      </c>
+      <c r="D73" t="s">
+        <v>337</v>
+      </c>
+      <c r="E73" s="7">
+        <v>1</v>
+      </c>
+      <c r="F73" s="24" t="s">
         <v>330</v>
-      </c>
-      <c r="C73" t="s">
-        <v>338</v>
-      </c>
-      <c r="D73" t="s">
-        <v>340</v>
-      </c>
-      <c r="E73" s="7">
-        <v>1</v>
-      </c>
-      <c r="F73" s="24" t="s">
-        <v>333</v>
       </c>
       <c r="G73" s="6">
         <v>129</v>
@@ -3485,19 +3499,19 @@
     </row>
     <row r="78" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C78" t="s">
+        <v>295</v>
+      </c>
+      <c r="D78" t="s">
+        <v>297</v>
+      </c>
+      <c r="E78" s="7">
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
         <v>298</v>
-      </c>
-      <c r="D78" t="s">
-        <v>300</v>
-      </c>
-      <c r="E78" s="7">
-        <v>1</v>
-      </c>
-      <c r="F78" t="s">
-        <v>301</v>
       </c>
       <c r="G78" s="6">
         <v>18.28</v>
@@ -3509,19 +3523,19 @@
     </row>
     <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C79" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D79" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E79" s="7">
         <v>1</v>
       </c>
       <c r="F79" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="G79" s="6">
         <v>10.81</v>
@@ -3533,19 +3547,19 @@
     </row>
     <row r="80" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C80" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D80" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="E80" s="7">
         <v>1</v>
       </c>
       <c r="F80" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G80" s="6">
         <v>7.8</v>
@@ -3557,36 +3571,36 @@
     </row>
     <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="C81" t="s">
         <v>419</v>
       </c>
-      <c r="C81" t="s">
-        <v>422</v>
-      </c>
       <c r="D81" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="E81">
         <v>1</v>
       </c>
       <c r="F81" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="C82" t="s">
+        <v>317</v>
+      </c>
+      <c r="D82" t="s">
+        <v>318</v>
+      </c>
+      <c r="E82" s="7">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
         <v>319</v>
-      </c>
-      <c r="C82" t="s">
-        <v>320</v>
-      </c>
-      <c r="D82" t="s">
-        <v>321</v>
-      </c>
-      <c r="E82" s="7">
-        <v>1</v>
-      </c>
-      <c r="F82" t="s">
-        <v>322</v>
       </c>
       <c r="G82" s="6">
         <v>2.19</v>
@@ -3598,19 +3612,19 @@
     </row>
     <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="C83" t="s">
+        <v>309</v>
+      </c>
+      <c r="D83" t="s">
+        <v>310</v>
+      </c>
+      <c r="E83" s="7">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
         <v>311</v>
-      </c>
-      <c r="C83" t="s">
-        <v>312</v>
-      </c>
-      <c r="D83" t="s">
-        <v>313</v>
-      </c>
-      <c r="E83" s="7">
-        <v>1</v>
-      </c>
-      <c r="F83" t="s">
-        <v>314</v>
       </c>
       <c r="G83" s="6">
         <v>3.51</v>
@@ -3622,13 +3636,13 @@
     </row>
     <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="C84" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="D84" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="E84" s="7">
         <v>16</v>
@@ -4161,16 +4175,16 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="B1" s="26" t="s">
         <v>136</v>
       </c>
       <c r="C1" s="33" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F1" t="s">
         <v>138</v>
@@ -4205,35 +4219,35 @@
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="31" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C2" s="34">
         <v>28</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="C3" s="34">
         <v>1</v>
       </c>
       <c r="D3" s="28" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="29" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B4" s="30" t="s">
         <v>155</v>
@@ -4242,12 +4256,12 @@
         <v>2</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="29" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B5" s="30" t="s">
         <v>179</v>
@@ -4256,12 +4270,12 @@
         <v>2</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="B6" s="30" t="s">
         <v>179</v>
@@ -4270,7 +4284,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -4284,12 +4298,12 @@
         <v>1</v>
       </c>
       <c r="D7" s="28" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" s="32" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B8" s="30" t="s">
         <v>179</v>
@@ -4298,12 +4312,12 @@
         <v>24</v>
       </c>
       <c r="D8" s="30" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B9" s="30" t="s">
         <v>179</v>
@@ -4312,7 +4326,7 @@
         <v>4</v>
       </c>
       <c r="D9" s="30" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -4326,12 +4340,12 @@
         <v>1</v>
       </c>
       <c r="D10" s="30" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B11" s="28" t="s">
         <v>179</v>
@@ -4340,7 +4354,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="28" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -4354,7 +4368,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="28" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -4368,12 +4382,12 @@
         <v>1</v>
       </c>
       <c r="D13" s="30" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="27" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B14" s="28" t="s">
         <v>149</v>
@@ -4387,7 +4401,7 @@
     </row>
     <row r="15" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A15" s="32" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="B15" s="30" t="s">
         <v>158</v>
@@ -4396,12 +4410,12 @@
         <v>16</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="27" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B16" s="28" t="s">
         <v>184</v>
@@ -4438,7 +4452,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -4446,13 +4460,13 @@
         <v>182</v>
       </c>
       <c r="B19" s="30" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C19" s="35">
         <v>1</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -4480,7 +4494,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -4494,7 +4508,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="30" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -4508,12 +4522,12 @@
         <v>1</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="27" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B24" s="28" t="s">
         <v>157</v>
@@ -4536,12 +4550,12 @@
         <v>1</v>
       </c>
       <c r="D25" s="28" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="27" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="B26" s="28" t="s">
         <v>73</v>
@@ -4550,7 +4564,7 @@
         <v>1</v>
       </c>
       <c r="D26" s="28" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -4564,12 +4578,12 @@
         <v>1</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="29" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="B28" s="30" t="s">
         <v>151</v>
@@ -4583,30 +4597,30 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="29" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C29" s="35">
         <v>1</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="29" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B30" s="30" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C30" s="35">
         <v>1</v>
       </c>
       <c r="D30" s="30" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -4620,7 +4634,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="28" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>